<commit_message>
Updated repo name in code
</commit_message>
<xml_diff>
--- a/Zinc/4. Exploratory data analysis/Inherent_characteristics_summary.xlsx
+++ b/Zinc/4. Exploratory data analysis/Inherent_characteristics_summary.xlsx
@@ -6,10 +6,10 @@
     <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="11370" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
-    <sheet name="Sites by type" sheetId="17" state="visible" r:id="rId1"/>
-    <sheet name="Sites by regime" sheetId="18" state="visible" r:id="rId2"/>
-    <sheet name="Sites by development" sheetId="19" state="visible" r:id="rId3"/>
-    <sheet name="Sites retained" sheetId="20" state="visible" r:id="rId4"/>
+    <sheet name="Sites by type" sheetId="21" state="visible" r:id="rId1"/>
+    <sheet name="Sites by regime" sheetId="22" state="visible" r:id="rId2"/>
+    <sheet name="Sites by development" sheetId="23" state="visible" r:id="rId3"/>
+    <sheet name="Sites retained" sheetId="24" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>

</xml_diff>